<commit_message>
feat: CATDUMB-style review card (HTML/CSS+Playwright) + caption grounding
- card/: self-contained renderer (template+fonts) ported from image-text-overlay skill
- review.py: render card instead of PIL overlay (PIL kept as fallback),
  ground caption/hook prompts (no invented scarcity/health claims),
  skip rows with invalid image_url
- review.yml: install playwright chromium
- review_products.xlsx: remove placeholder row

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/review_products.xlsx
+++ b/review_products.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="630" yWindow="615" windowWidth="37095" windowHeight="17310" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G144"/>
+  <dimension ref="A1:G143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -522,41 +522,10 @@
       </c>
     </row>
     <row r="2" ht="39.95" customHeight="1">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>วางรายละเอียดสินค้าจาก Shopee ทั้งหมดที่นี่</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>https://s.lazada.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://down-th.img.susercontent.com/xxx.jpg</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>ลด 20%</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="345" customHeight="1">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>RAY-BAN JUSTIN- RB4165F 601/71
 Ray-Ban เรแบนเป็นผู้นำด้านการผลิตแว่นกันแดด และแว่นสายตา ที่ได้ความนิยมมากที่สุดทั่วโลก มีให้เลือกหลากหลายสไตล์ เหมาะกับทุกคน และใส่ได้ทั้งผู้หญิงและผู้ชาย
@@ -570,23 +539,23 @@
 Lens Material: Polycarbonate Standard</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>https://s.shopee.co.th/AUqz80oxUd</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>https://s.lazada.co.th/s.Z6PzJE?c=b&amp;t=p-ijr1Q-svKWG</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>https://down-th.img.susercontent.com/file/th-11134201-7r990-lscec08f21gm73.webp
 https://down-th.img.susercontent.com/file/th-11134201-7r98y-lscec0amysmu78.webp</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">฿5,130
 final price indicator icon
@@ -598,17 +567,17 @@
 </t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>done 2026-05-21 13:15</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="409.5" customHeight="1">
-      <c r="A4" t="n">
+    <row r="3" ht="345" customHeight="1">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Sony BRAVIA 3 ทีวี 55 นิ้ว รุ่น K-55S30 4K Ultra HD Smart TV (Google TV) | 4K HDR Processor X1
 รายละเอียดสินค้า
@@ -628,22 +597,22 @@
 เรียกดูภาพยนตร์และรายการทีวีมากกว่า 400,000 ตอนจากบริการสตรีมมิ่งของคุณทั้งหมดในที่เดียว โดยจัดเป็นหัวข้อและแนวเนื้อหาไว้ตามสิ่งที่คุณสนใจ</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>https://s.shopee.co.th/10zvLKc6Ji</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>https://s.lazada.co.th/s.Z6mEyG?c=a&amp;t=p-i0-s0&amp;sub_id1=W1</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>https://down-th.img.susercontent.com/file/th-11134207-7r98v-lvsn9yh5vql9c5.webp</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">฿20,500
 final price indicator icon
@@ -653,129 +622,154 @@
 </t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>done 2026-05-31 16:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="409.5" customHeight="1">
+      <c r="A4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Benefruit มะพร้าวอบแห้ง🥥 มะพร้าวกรอบ เนื้อแน่นกรึบ หวานน้อย สูตรน้ำตาลต่ำ (Dried Coconut) ราคา 189.00 บาท</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3qKMKSQPB2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mg3ydny6nkzwa4.webp</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>done 2026-05-31 16:19</t>
+          <t>done 2026-06-05 11:44</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Benefruit มะพร้าวอบแห้ง🥥 มะพร้าวกรอบ เนื้อแน่นกรึบ หวานน้อย สูตรน้ำตาลต่ำ (Dried Coconut) ราคา 189.00 บาท</t>
+          <t>เก๊กฮวยผงสำเร็จรูป HighlandHerb ขนาด 600 กรัม ราคา 249.00 บาท</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qKMKSQPB2</t>
+          <t>https://s.shopee.co.th/3VhVvoUPHl</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mg3ydny6nkzwa4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98v-lp4vdgeuw77id2.webp</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>done 2026-06-05 11:44</t>
+          <t>done 2026-06-05 11:57</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>เก๊กฮวยผงสำเร็จรูป HighlandHerb ขนาด 600 กรัม ราคา 249.00 บาท</t>
+          <t>❤️ส่งด่วน1วัน รีวิวเยอะสุด 🙏เกรดพรีเมี่ยม ทุเรียนหมอนทองจันทบุรี แกะเนื้อล้วน พร้อมทาน 🚚ส่งรถเย็น ราคา 469.00 บาท</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3VhVvoUPHl</t>
+          <t>https://s.shopee.co.th/1gFrkSHnnm</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98v-lp4vdgeuw77id2.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0o-mcoacmrgvbz293.webp</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>done 2026-06-05 11:57</t>
+          <t>done 2026-06-05 22:49</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>❤️ส่งด่วน1วัน รีวิวเยอะสุด 🙏เกรดพรีเมี่ยม ทุเรียนหมอนทองจันทบุรี แกะเนื้อล้วน พร้อมทาน 🚚ส่งรถเย็น ราคา 469.00 บาท</t>
+          <t>ชาเขียว 100% เพียวมัทฉะ ชาเขียว พรีเมี่ยม matcha powder from japan 0 สารเติมแต่ง 1 กระป๋อง 300g ราคา 374.00 บาท</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1gFrkSHnnm</t>
+          <t>https://s.shopee.co.th/1qZHwlPy1j</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0o-mcoacmrgvbz293.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mhivoyzzzqird0.webp</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>done 2026-06-05 22:49</t>
+          <t>done 2026-06-06 09:30</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ชาเขียว 100% เพียวมัทฉะ ชาเขียว พรีเมี่ยม matcha powder from japan 0 สารเติมแต่ง 1 กระป๋อง 300g ราคา 374.00 บาท</t>
+          <t>ไส้อั่วโฮมเมดสูตรเชียงใหม่ หอมสมุนไพร เครื่องแกงเราทำเอง ชุด2แพ็ค รวมน้ำหนัก 1กิโลกรัม ราคา 337.00 บาท</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1qZHwlPy1j</t>
+          <t>https://s.shopee.co.th/2qS1GCKbXS</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mhivoyzzzqird0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/0b788de026956cdf22390697e7a0306c.webp</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>done 2026-06-06 09:30</t>
+          <t>done 2026-06-08 05:46</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ไส้อั่วโฮมเมดสูตรเชียงใหม่ หอมสมุนไพร เครื่องแกงเราทำเอง ชุด2แพ็ค รวมน้ำหนัก 1กิโลกรัม ราคา 337.00 บาท</t>
+          <t>ทุเรียนจันทบุรีเนื้อพรีเมียม ยอดขายเยอะที่สุดทุเรียนหมอนทอง คัดเนื้อเทพไม่เน้นทรง เนื้อเหลือง เนื้อตลาดที่คนไทยกิน ราคา 621.00 บาท</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qS1GCKbXS</t>
+          <t>https://s.shopee.co.th/5fmCd5ZUob</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/0b788de026956cdf22390697e7a0306c.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rask-mabmx8hshx6278.webp</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -786,21 +780,21 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ทุเรียนจันทบุรีเนื้อพรีเมียม ยอดขายเยอะที่สุดทุเรียนหมอนทอง คัดเนื้อเทพไม่เน้นทรง เนื้อเหลือง เนื้อตลาดที่คนไทยกิน ราคา 621.00 บาท</t>
+          <t>หมูกรอบ เงินล้าน เนื้อเยอะ มันน้อย เนื้อแน่น หนังกรอบ กรอบนอกนุ่มใน พร้อมน้ำจิ้ม ขนาด 500ก./ 1,000ก. ราคา 290.00 บาท</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5fmCd5ZUob</t>
+          <t>https://s.shopee.co.th/7pqf9H2jLU</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rask-mabmx8hshx6278.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rask-m76elywra3an63.webp</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -811,21 +805,21 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>หมูกรอบ เงินล้าน เนื้อเยอะ มันน้อย เนื้อแน่น หนังกรอบ กรอบนอกนุ่มใน พร้อมน้ำจิ้ม ขนาด 500ก./ 1,000ก. ราคา 290.00 บาท</t>
+          <t>กุ้งจ่อมโคราชแท้ 100% ขนาด 500 กรัม (ส่งตรงจากบ้านปลาจ่อม อำเภอปักธงชัย จังหวัดนครราชสีมา) ราคา 90.00 บาท</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7pqf9H2jLU</t>
+          <t>https://s.shopee.co.th/6VLJcuyatD</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rask-m76elywra3an63.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/0952cbb174eccbe472d21bbfd74f6b1e.webp</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -836,21 +830,21 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>กุ้งจ่อมโคราชแท้ 100% ขนาด 500 กรัม (ส่งตรงจากบ้านปลาจ่อม อำเภอปักธงชัย จังหวัดนครราชสีมา) ราคา 90.00 บาท</t>
+          <t>[แพ็คเกจลุ้นรางวัล][แพ็ค 6] Tulip Cocoa Powder Dark Brown Colour 440 g. ทิวลิปผงโกโก้สีเข้ม 440 กรัม ราคา 1335.00 บาท</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6VLJcuyatD</t>
+          <t>https://s.shopee.co.th/BRG53bISA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/0952cbb174eccbe472d21bbfd74f6b1e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823pw-mowwmk8cx5vmdc.webp</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -861,46 +855,46 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[แพ็คเกจลุ้นรางวัล][แพ็ค 6] Tulip Cocoa Powder Dark Brown Colour 440 g. ทิวลิปผงโกโก้สีเข้ม 440 กรัม ราคา 1335.00 บาท</t>
+          <t>ขายดี🔥 Benefruit ส้มอบแห้ง🍊ส้มหนึบ กลีบส้ม ไร้เม็ด ผลไม้อบแห้งเกรดส่งออก สูตรน้ำตาลต่ำ (Dried Orange Low Sugar) ราคา 95.00 บาท</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/BRG53bISA</t>
+          <t>https://s.shopee.co.th/6fehl9kz4K</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823pw-mowwmk8cx5vmdc.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m6tjad8k1fxc38.webp</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>done 2026-06-08 05:46</t>
+          <t>done 2026-06-08 07:40</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ขายดี🔥 Benefruit ส้มอบแห้ง🍊ส้มหนึบ กลีบส้ม ไร้เม็ด ผลไม้อบแห้งเกรดส่งออก สูตรน้ำตาลต่ำ (Dried Orange Low Sugar) ราคา 95.00 บาท</t>
+          <t>ขนมเปี๊ยะลาวาไส้ฝอยทองนูเทลล่า (350g) Noeyleeshop ราคา 94.00 บาท</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6fehl9kz4K</t>
+          <t>https://s.shopee.co.th/8fPoCgrCHw</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m6tjad8k1fxc38.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasb-mb1xybwmbxc1d2.webp</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -911,46 +905,46 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ขนมเปี๊ยะลาวาไส้ฝอยทองนูเทลล่า (350g) Noeyleeshop ราคา 94.00 บาท</t>
+          <t>หมูหวานซีอิ๊วงา ทอดไท (นุ่ม-ไม่แข็ง 150 ก) 👉 ไม่ใส่พริกไทย เด็กทานได้ ราคา 114.00 บาท</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8fPoCgrCHw</t>
+          <t>https://s.shopee.co.th/110N4eA1qB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasb-mb1xybwmbxc1d2.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98y-lr10flflzagt5a.webp</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>done 2026-06-08 07:40</t>
+          <t>done 2026-06-08 07:41</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>หมูหวานซีอิ๊วงา ทอดไท (นุ่ม-ไม่แข็ง 150 ก) 👉 ไม่ใส่พริกไทย เด็กทานได้ ราคา 114.00 บาท</t>
+          <t>นมกล่อง (ยกลัง) นมยูเอชที นมไฮคิวสูตร3 1พลัส ซูเปอร์โกลด์ รสจืด180 มล (27 กล่อง) นม UHT HiQ Super Gold UHT ราคา 669.00 บาท</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/110N4eA1qB</t>
+          <t>https://s.shopee.co.th/2qS1FunWwa</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98y-lr10flflzagt5a.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasg-m7hrtewsksjj0d.webp</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -961,21 +955,21 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>นมกล่อง (ยกลัง) นมยูเอชที นมไฮคิวสูตร3 1พลัส ซูเปอร์โกลด์ รสจืด180 มล (27 กล่อง) นม UHT HiQ Super Gold UHT ราคา 669.00 บาท</t>
+          <t>น้ำมันปาล์ม ตรา หยก ขนาด1ลิตร แพ็ค 3 ขวด ราคา 210.00 บาท</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qS1FunWwa</t>
+          <t>https://s.shopee.co.th/70HaDgeSt4</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasg-m7hrtewsksjj0d.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823rr-mp0ouarhqkn61b.webp</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -986,46 +980,46 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>น้ำมันปาล์ม ตรา หยก ขนาด1ลิตร แพ็ค 3 ขวด ราคา 210.00 บาท</t>
+          <t>ขนมอัลมอนด์ดาร์กช็อค ไม่ใส่เนย ไม่ใส่แป้ง Ketoทานได้ สูตรคลีนเพื่อสุขภาพ Almond DarkChoc Kanomdeedee (ขนมดีดี) ราคา 193.00 บาท</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/70HaDgeSt4</t>
+          <t>https://s.shopee.co.th/8pjEP3FPCX</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823rr-mp0ouarhqkn61b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mjlfxs2zdmva1c.webp</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>done 2026-06-08 07:41</t>
+          <t>done 2026-06-09 06:03</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ขนมอัลมอนด์ดาร์กช็อค ไม่ใส่เนย ไม่ใส่แป้ง Ketoทานได้ สูตรคลีนเพื่อสุขภาพ Almond DarkChoc Kanomdeedee (ขนมดีดี) ราคา 193.00 บาท</t>
+          <t>[ของแท้ ต้นตำรับ] หยิบเป็นชิ้นทานง่าย หมี่กรอบเตาถ่าน กรอบนุ่มไม่แข็ง หอมผิวส้มซ่า (1กล่อง 60 ชิ้น) ราคา 251.00 บาท</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8pjEP3FPCX</t>
+          <t>https://s.shopee.co.th/4qD5devtq4</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mjlfxs2zdmva1c.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mlth9szef6df1f.webp</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1036,21 +1030,21 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[ของแท้ ต้นตำรับ] หยิบเป็นชิ้นทานง่าย หมี่กรอบเตาถ่าน กรอบนุ่มไม่แข็ง หอมผิวส้มซ่า (1กล่อง 60 ชิ้น) ราคา 251.00 บาท</t>
+          <t>น้ำพริกกากหมู ขนาด 150 กรัม แบบกระปุก แซ่บปะล้ำปะเหลือ ราคา 158.00 บาท</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4qD5devtq4</t>
+          <t>https://s.shopee.co.th/17psx9vPd</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mlth9szef6df1f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul6-lig9ntju66lk6e.webp</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1061,46 +1055,46 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>น้ำพริกกากหมู ขนาด 150 กรัม แบบกระปุก แซ่บปะล้ำปะเหลือ ราคา 158.00 บาท</t>
+          <t>ค่าส่งถูกที่สุดร้านช่วยจ่าย ยอดขายเยอะที่สุดทุเรียนหมอนทอง คัดเนื้อเทพไม่เน้นทรง เนื้อเหลือง เนื้อตลาดที่คนไทยกิน ราคา 621.00 บาท</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/17psx9vPd</t>
+          <t>https://s.shopee.co.th/4ftfRK3fOI</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qul6-lig9ntju66lk6e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r992-lx9x2ueokgxcc9.webp</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>done 2026-06-09 06:03</t>
+          <t>done 2026-06-09 06:04</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ค่าส่งถูกที่สุดร้านช่วยจ่าย ยอดขายเยอะที่สุดทุเรียนหมอนทอง คัดเนื้อเทพไม่เน้นทรง เนื้อเหลือง เนื้อตลาดที่คนไทยกิน ราคา 621.00 บาท</t>
+          <t>น้ำพริกกากหมู ยาหยี (200 ก) 🌶 อร่อย 🔥มีเนื้อ - มีหนัง ราคา 99.00 บาท</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4ftfRK3fOI</t>
+          <t>https://s.shopee.co.th/4ftfRbjCEv</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r992-lx9x2ueokgxcc9.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98q-lr8le588wcsd92.webp</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1111,46 +1105,46 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>น้ำพริกกากหมู ยาหยี (200 ก) 🌶 อร่อย 🔥มีเนื้อ - มีหนัง ราคา 99.00 บาท</t>
+          <t>เมล็ดกาแฟคั่ว เขาทะลุ ชุมพร💥คัดเกรดขนาด 500 กรัม กาแฟโรบัสต้า จากขุนเขาชุมพร สู่กาแฟพรีเมียมไทย | Khao Thalu Coffee ราคา 180.00 บาท</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4ftfRbjCEv</t>
+          <t>https://s.shopee.co.th/6VLJciC5w7</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98q-lr8le588wcsd92.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mjh2qiig3y83e1.webp</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>done 2026-06-09 06:04</t>
+          <t>done 2026-06-10 06:04</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>เมล็ดกาแฟคั่ว เขาทะลุ ชุมพร💥คัดเกรดขนาด 500 กรัม กาแฟโรบัสต้า จากขุนเขาชุมพร สู่กาแฟพรีเมียมไทย | Khao Thalu Coffee ราคา 180.00 บาท</t>
+          <t>ปลาหมึกไข่แดดเดียวทอดพร้อมทาน -(ไข่ทุกตัว) ไซร์ 5-9 ตัวต่อแพค น้ำหนักก่อนทอด300กรัมและ 500 กรัม ราคา 325.00 บาท</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6VLJciC5w7</t>
+          <t>https://s.shopee.co.th/6fehlA2J9M</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mjh2qiig3y83e1.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/23e49a44f577b0531100e55e0851f11f.webp</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1161,21 +1155,21 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ปลาหมึกไข่แดดเดียวทอดพร้อมทาน -(ไข่ทุกตัว) ไซร์ 5-9 ตัวต่อแพค น้ำหนักก่อนทอด300กรัมและ 500 กรัม ราคา 325.00 บาท</t>
+          <t>[โปร 3 กระปุก] น้ำพริกแจ่วบอง ไร่จิตภักดี แบบผัดสุก รสชาติเผ็ดนัวแซ่บถึงใจ ขนาด150กรัม ราคา 219.00 บาท</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6fehlA2J9M</t>
+          <t>https://s.shopee.co.th/LkgHbeZU4</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/23e49a44f577b0531100e55e0851f11f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasc-m8x35mczvx0ude.webp</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1186,46 +1180,46 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>[โปร 3 กระปุก] น้ำพริกแจ่วบอง ไร่จิตภักดี แบบผัดสุก รสชาติเผ็ดนัวแซ่บถึงใจ ขนาด150กรัม ราคา 219.00 บาท</t>
+          <t>น้ำพริกปลาแซลมอน น้ำพริกรสแซ่บ น้ำพริกแห้ง ขนาด 80 กรัม แม่ทองคำรสแซ่บ แซลมอน Salmon Chilli Paste ราคา 55.00 บาท</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/LkgHbeZU4</t>
+          <t>https://s.shopee.co.th/9AM4ncO9EF</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasc-m8x35mczvx0ude.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98p-lrzz1m8bd41pfb.webp</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>done 2026-06-10 06:04</t>
+          <t>done 2026-06-10 06:05</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>น้ำพริกปลาแซลมอน น้ำพริกรสแซ่บ น้ำพริกแห้ง ขนาด 80 กรัม แม่ทองคำรสแซ่บ แซลมอน Salmon Chilli Paste ราคา 55.00 บาท</t>
+          <t>ปังเปี๊ยะโมจินมสดฮอกไกโด250g แถมดริปนูเทลล่า 40g ราคา 79.00 บาท</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9AM4ncO9EF</t>
+          <t>https://s.shopee.co.th/9UyvCR64vP</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98p-lrzz1m8bd41pfb.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0g-mcltjs8w1rlsba.webp</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1236,46 +1230,46 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ปังเปี๊ยะโมจินมสดฮอกไกโด250g แถมดริปนูเทลล่า 40g ราคา 79.00 บาท</t>
+          <t>Chocolate Brownie Bite ช็อกโกแลตบราวนี่ไบท์ บราวนี่หน้าฟิล์ม ราคา 119.00 บาท</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9UyvCR64vP</t>
+          <t>https://s.shopee.co.th/4AxMmYCMnR</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0g-mcltjs8w1rlsba.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-23030-bggj3q1eovovda.webp</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>done 2026-06-10 06:05</t>
+          <t>done 2026-06-10 11:15</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Chocolate Brownie Bite ช็อกโกแลตบราวนี่ไบท์ บราวนี่หน้าฟิล์ม ราคา 119.00 บาท</t>
+          <t>ปลาหมึกแห้ง ปลาหมึกแพไข่ ไซส์กลาง ไม่เค็มมาก ตากสดใหม่ รับประกันความอร่อย ราคา 129.00 บาท</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4AxMmYCMnR</t>
+          <t>https://s.shopee.co.th/6pyA1F9Gqv</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-23030-bggj3q1eovovda.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-22110-pkze82odovjv1f.webp</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1286,21 +1280,21 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ปลาหมึกแห้ง ปลาหมึกแพไข่ ไซส์กลาง ไม่เค็มมาก ตากสดใหม่ รับประกันความอร่อย ราคา 129.00 บาท</t>
+          <t>Cheesy Jujube - พุทรานมชีส 250 กรัม ขนม อร่อย โฮมเมด นูกัตตี๋เล็ก พุทรา นม ชีส ของฝาก ขนมทานเล่น by teeleknougat ราคา 189.00 บาท</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6pyA1F9Gqv</t>
+          <t>https://s.shopee.co.th/8fPoCsmUHB</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-22110-pkze82odovjv1f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mgdl0qn5u70q1e.webp</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1311,46 +1305,46 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cheesy Jujube - พุทรานมชีส 250 กรัม ขนม อร่อย โฮมเมด นูกัตตี๋เล็ก พุทรา นม ชีส ของฝาก ขนมทานเล่น by teeleknougat ราคา 189.00 บาท</t>
+          <t>KETO ไส้อั่วหมูสมุนไพรคีโต ย่างหอมๆจากเมืองเหนือ คีโต-โลว์คาร์บทานได้ ราคา 109.00 บาท</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8fPoCsmUHB</t>
+          <t>https://s.shopee.co.th/17psy0rKS</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mgdl0qn5u70q1e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98r-ltgbf2j90fi721.webp</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>done 2026-06-10 11:15</t>
+          <t>done 2026-06-10 11:16</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>KETO ไส้อั่วหมูสมุนไพรคีโต ย่างหอมๆจากเมืองเหนือ คีโต-โลว์คาร์บทานได้ ราคา 109.00 บาท</t>
+          <t>(แบบไม่มีน้ำจิ้ม) หมูกรอบ อบ ไม่มีไขมันทรานส์ เนื้อนุ่ม หนังกรอบ by หมูกรอบ SNOOK ราคา 172.00 บาท</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/17psy0rKS</t>
+          <t>https://s.shopee.co.th/W46TxsKWN</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98r-ltgbf2j90fi721.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/cc8c958732c4728a5538bdd8ae6475f8.webp</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1361,71 +1355,71 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>(แบบไม่มีน้ำจิ้ม) หมูกรอบ อบ ไม่มีไขมันทรานส์ เนื้อนุ่ม หนังกรอบ by หมูกรอบ SNOOK ราคา 172.00 บาท</t>
+          <t>หมูแดดเดียวพรีเมียม อบลมร้อน สะอาด ไร้ฝุ่น ไร้แมลง เนื้อนุ่ม ฉ่ำ ทอดง่าย ราคา 149.00 บาท</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/W46TxsKWN</t>
+          <t>https://s.shopee.co.th/30lRSKFxR4</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/cc8c958732c4728a5538bdd8ae6475f8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mm8rnpzzshs429.webp</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>done 2026-06-10 11:16</t>
+          <t>done 2026-06-11 06:14</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>หมูแดดเดียวพรีเมียม อบลมร้อน สะอาด ไร้ฝุ่น ไร้แมลง เนื้อนุ่ม ฉ่ำ ทอดง่าย ราคา 149.00 บาท</t>
+          <t>ผงชาเขียวอาโอโมริ"AOMORI Matcha"ผงชาเขียวมัทฉะ 100% สูตรพรีเมี่ยม 100g. ราคา 119.00 บาท</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/30lRSKFxR4</t>
+          <t>https://s.shopee.co.th/1LdDTGYsoS</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mm8rnpzzshs429.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m5sqf6g4v4c668.webp</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>done 2026-06-11 06:14</t>
+          <t>done 2026-06-11 06:15</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ผงชาเขียวอาโอโมริ"AOMORI Matcha"ผงชาเขียวมัทฉะ 100% สูตรพรีเมี่ยม 100g. ราคา 119.00 บาท</t>
+          <t>น้ำพริกหนังไก่ ยาหยี (100/150/200 ก) 🌶 เผ็ด จัดจ้าน ราคา 75.00 บาท</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1LdDTGYsoS</t>
+          <t>https://s.shopee.co.th/50WTm4WhFs</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m5sqf6g4v4c668.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r991-lr10flflv2rh60.webp</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1436,21 +1430,21 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>น้ำพริกหนังไก่ ยาหยี (100/150/200 ก) 🌶 เผ็ด จัดจ้าน ราคา 75.00 บาท</t>
+          <t>เบนิฟิตต์ ไฮโปรตีน ขนาด350 มล.( หมดอายุ เดือน 9-10/2026)จัดส่งภายใน2-3วัน(สั่ง1ลังต่อคำสั่งซื้อ) ราคา 399.00 บาท</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/50WTm4WhFs</t>
+          <t>https://s.shopee.co.th/3LOHr6tssA</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r991-lr10flflv2rh60.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mlh91o6kf95bed.webp</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1461,21 +1455,21 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>เบนิฟิตต์ ไฮโปรตีน ขนาด350 มล.( หมดอายุ เดือน 9-10/2026)จัดส่งภายใน2-3วัน(สั่ง1ลังต่อคำสั่งซื้อ) ราคา 399.00 บาท</t>
+          <t>เม็ดมะม่วงหิมพานต์อบ 500 กรัม เกรด A เต็มเม็ด หอม กรอบ ไม่ทอด | Khunja Shop ราคา 155.00 บาท</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3LOHr6tssA</t>
+          <t>https://s.shopee.co.th/9AM4nb7QzA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mlh91o6kf95bed.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zti-miibfjkeai2q55.webp</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1486,26 +1480,26 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>เม็ดมะม่วงหิมพานต์อบ 500 กรัม เกรด A เต็มเม็ด หอม กรอบ ไม่ทอด | Khunja Shop ราคา 155.00 บาท</t>
+          <t>ตราฉัตร 5 กิโล ข้าวหอมมะลิใหม่ ข้าวหอมมะลิแท้ ตราฉัตร 5kg. (หอม นุ่ม ตลอดปี) ข้าวหอมผสม ข้าวขาว หุงอร่อย หุงขึ้นหม้อ ราคา 134.00 บาท</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9AM4nb7QzA</t>
+          <t>https://s.shopee.co.th/2qRzC7LIj7</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zti-miibfjkeai2q55.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-8260m-mkdsz738rxtu0a.webp</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>done 2026-06-11 06:15</t>
+          <t>done 2026-06-12 06:11</t>
         </is>
       </c>
     </row>
@@ -1515,17 +1509,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ตราฉัตร 5 กิโล ข้าวหอมมะลิใหม่ ข้าวหอมมะลิแท้ ตราฉัตร 5kg. (หอม นุ่ม ตลอดปี) ข้าวหอมผสม ข้าวขาว หุงอร่อย หุงขึ้นหม้อ ราคา 134.00 บาท</t>
+          <t>ผลไม้ดอง 1kg บรรจุขวดโหล ชั่งเฉพาะเนื้อ แถมฟรีพริกเกลือรสเด็ด ราคา 100.00 บาท</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qRzC7LIj7</t>
+          <t>https://s.shopee.co.th/7fXH0vfIv3</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-8260m-mkdsz738rxtu0a.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-ll6odn47bqr032.webp</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1536,21 +1530,21 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ผลไม้ดอง 1kg บรรจุขวดโหล ชั่งเฉพาะเนื้อ แถมฟรีพริกเกลือรสเด็ด ราคา 100.00 บาท</t>
+          <t>น้ำพริกหมูกระจกมะเดี่ยว วับวาว รสต้มยำ ชิ้นใหญ่ เต็มคำ แซ่บ เปรี้ยวเผ็ดสะใจ มี2ขนาด 100g./400g. ราคา 177.00 บาท</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7fXH0vfIv3</t>
+          <t>https://s.shopee.co.th/8pjCL6ho1X</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-ll6odn47bqr032.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mnmij2prwhl2a7.webp</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1561,21 +1555,21 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>น้ำพริกหมูกระจกมะเดี่ยว วับวาว รสต้มยำ ชิ้นใหญ่ เต็มคำ แซ่บ เปรี้ยวเผ็ดสะใจ มี2ขนาด 100g./400g. ราคา 177.00 บาท</t>
+          <t>ผงมัทฉะ ออร์แกนิค 100% กลิ่นหอมละมุน ชงง่ายในทุกเมนู - RAIWAN ขนาด 100 กรัม ราคา 340.00 บาท</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8pjCL6ho1X</t>
+          <t>https://s.shopee.co.th/30lPOOyjCD</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mnmij2prwhl2a7.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0s-md4csnzellfp52.webp</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1586,21 +1580,21 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ผงมัทฉะ ออร์แกนิค 100% กลิ่นหอมละมุน ชงง่ายในทุกเมนู - RAIWAN ขนาด 100 กรัม ราคา 340.00 บาท</t>
+          <t>น้ำพริกปูม้า แบรนด์ บังฟิส มันปู/ไข่ปู/เนื้อปู ราคา 169.00 บาท</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/30lPOOyjCD</t>
+          <t>https://s.shopee.co.th/4AxOqi9zhi</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0s-md4csnzellfp52.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98v-lzsvhmsql75t87.webp</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1611,46 +1605,46 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>น้ำพริกปูม้า แบรนด์ บังฟิส มันปู/ไข่ปู/เนื้อปู ราคา 169.00 บาท</t>
+          <t>ปุยแสบปาก พริกผัดน้ำมันมะกอก Vegen ราคา 263.00 บาท</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4AxOqi9zhi</t>
+          <t>https://s.shopee.co.th/AKY2C1mROs</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98v-lzsvhmsql75t87.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mnu2gil3c16u83.webp</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>done 2026-06-12 06:11</t>
+          <t>done 2026-06-13 06:03</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ปุยแสบปาก พริกผัดน้ำมันมะกอก Vegen ราคา 263.00 บาท</t>
+          <t>ส่งด่วนกรุงเทพ/ตจว.❤️ทุเรียนหมอนทองระยอง-จัน แท้💯พรีเมี่ยม แกะเนื้อ รับประกันไม่ตรงปกเปลี่ยนใหม่ให้100%💋 ส่งทุกวัน ราคา 415.00 บาท</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AKY2C1mROs</t>
+          <t>https://s.shopee.co.th/9fILOaKtZ4</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mnu2gil3c16u83.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mkjkqzprk3ye45.webp</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1661,21 +1655,21 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ส่งด่วนกรุงเทพ/ตจว.❤️ทุเรียนหมอนทองระยอง-จัน แท้💯พรีเมี่ยม แกะเนื้อ รับประกันไม่ตรงปกเปลี่ยนใหม่ให้100%💋 ส่งทุกวัน ราคา 415.00 บาท</t>
+          <t>[เซ็ตคู่] น้ำพริกไข่ปูม้า + น้ำพริกเนื้อปูม้า น้ำพริก ปูม้ามีเลขฮาลาลทุกสูตร . ราคา 304.00 บาท</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fILOaKtZ4</t>
+          <t>https://s.shopee.co.th/5Apw2WWZJu</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mkjkqzprk3ye45.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasi-m5phpwu6gkvqac.webp</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1686,46 +1680,46 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>[เซ็ตคู่] น้ำพริกไข่ปูม้า + น้ำพริกเนื้อปูม้า น้ำพริก ปูม้ามีเลขฮาลาลทุกสูตร . ราคา 304.00 บาท</t>
+          <t>[Official] 🔥 [KETO] Wholesweet น้ำเชื่อมหญ้าหวาน ไซรัปหญ้าหวาน สูตรคีโต 320 มล. ราคา 151.00 บาท</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5Apw2WWZJu</t>
+          <t>https://s.shopee.co.th/1BJnH6JRHT</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasi-m5phpwu6gkvqac.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/a59d309f9d3e34b88669ec977426484d.webp</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>done 2026-06-13 06:03</t>
+          <t>done 2026-06-13 06:04</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>[Official] 🔥 [KETO] Wholesweet น้ำเชื่อมหญ้าหวาน ไซรัปหญ้าหวาน สูตรคีโต 320 มล. ราคา 151.00 บาท</t>
+          <t>หมูแดดเดียว หมูเบทาโกรเกรดA ไม่ใส่สารกันบูด ไม่เหนียว ไม่แข็ง สีธรรมชาติ วัตถุดิบเครื่องปรุงคุณภาพสูง อร่อย สะอาด มี อย. ราคา 92.00 บาท</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1BJnH6JRHT</t>
+          <t>https://s.shopee.co.th/5Apw2XRyH1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/a59d309f9d3e34b88669ec977426484d.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-lxflamy6285r9b.webp</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -1736,26 +1730,26 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>หมูแดดเดียว หมูเบทาโกรเกรดA ไม่ใส่สารกันบูด ไม่เหนียว ไม่แข็ง สีธรรมชาติ วัตถุดิบเครื่องปรุงคุณภาพสูง อร่อย สะอาด มี อย. ราคา 92.00 บาท</t>
+          <t>(แพ็ค 24 ซอง) Muek Groob หมึกกรุบ เส้นบุกปรุงรสหม่าล่า (เลือกรสชาติได้) ราคา 532.00 บาท</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5Apw2XRyH1</t>
+          <t>https://s.shopee.co.th/1gG3rjy0Kb</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-lxflamy6285r9b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mp4md3z4eyvi66.webp</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>done 2026-06-13 06:04</t>
+          <t>done 2026-06-14 05:45</t>
         </is>
       </c>
     </row>
@@ -1765,42 +1759,42 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>(แพ็ค 24 ซอง) Muek Groob หมึกกรุบ เส้นบุกปรุงรสหม่าล่า (เลือกรสชาติได้) ราคา 532.00 บาท</t>
+          <t>ขายดีมาก ปลาสลิดไข่ 4-5 ตัว 500 กรัม📌(ซื้อ2แพคคุ้มกว่าจ้า) เค็มน้อย อร่อยมาก มีไข่จุกๆทุกตัว ราคา 200.00 บาท</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1gG3rjy0Kb</t>
+          <t>https://s.shopee.co.th/7pqhDM2ExP</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mp4md3z4eyvi66.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mg3tpwy77v2m4b.webp</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>done 2026-06-14 05:45</t>
+          <t>done 2026-06-14 05:46</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ขายดีมาก ปลาสลิดไข่ 4-5 ตัว 500 กรัม📌(ซื้อ2แพคคุ้มกว่าจ้า) เค็มน้อย อร่อยมาก มีไข่จุกๆทุกตัว ราคา 200.00 บาท</t>
+          <t>Llamito ผงมัทฉะ ออร์แกนิค (Matcha Powder) ขนาด 250g ราคา 449.00 บาท</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7pqhDM2ExP</t>
+          <t>https://s.shopee.co.th/qgwsYVoHw</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mg3tpwy77v2m4b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mih9x5ddqn0n95.webp</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -1815,17 +1809,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Llamito ผงมัทฉะ ออร์แกนิค (Matcha Powder) ขนาด 250g ราคา 449.00 บาท</t>
+          <t>อุดมสุข น้ำพริกอกไก่คลีน น้ำพริกอกไก่ น้ำพริกคลีน น้ำพริกคีโต อาหารเพื่อสุขภาพ อาหารคลีน อาหารคีโต ราคา 109.00 บาท</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/qgwsYVoHw</t>
+          <t>https://s.shopee.co.th/5VSmQmR3XO</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mih9x5ddqn0n95.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mgdp5aurnthl96.webp</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -1836,21 +1830,21 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>อุดมสุข น้ำพริกอกไก่คลีน น้ำพริกอกไก่ น้ำพริกคลีน น้ำพริกคีโต อาหารเพื่อสุขภาพ อาหารคลีน อาหารคีโต ราคา 109.00 บาท</t>
+          <t>เต้าหู้เฮียแว่น เต้าหู้เนื้อครีมคัสตาร์ด กรอบนอก ครีมฉ่ำ นิ่มละมุน | แพ็ค 5 ชิ้น 1 กิโล | โปรตีน 55 กรัม | แช่เย็น 7 วัน ราคา 175.00 บาท</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5VSmQmR3XO</t>
+          <t>https://s.shopee.co.th/1BJnGwvqq6</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mgdp5aurnthl96.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-ml3bpvzk2l8ic2.webp</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -1861,46 +1855,46 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>เต้าหู้เฮียแว่น เต้าหู้เนื้อครีมคัสตาร์ด กรอบนอก ครีมฉ่ำ นิ่มละมุน | แพ็ค 5 ชิ้น 1 กิโล | โปรตีน 55 กรัม | แช่เย็น 7 วัน ราคา 175.00 บาท</t>
+          <t>(6.6) koreadong โคเรียดอง 4 กระปุก แซลมอน 2 กุ้ง 2 ฟรี!! น้ำจิ้ม 2 สูตร ราคา 1089.00 บาท</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1BJnGwvqq6</t>
+          <t>https://s.shopee.co.th/6VLJcekMgd</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-ml3bpvzk2l8ic2.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mp3lp4rqcflt1c.webp</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>done 2026-06-14 05:46</t>
+          <t>done 2026-06-15 05:50</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>(6.6) koreadong โคเรียดอง 4 กระปุก แซลมอน 2 กุ้ง 2 ฟรี!! น้ำจิ้ม 2 สูตร ราคา 1089.00 บาท</t>
+          <t>koreadong โคเรียดอง แซลมอนดองซีอิ๊วเกาหลี 1 กระปุก ขนาด 500 กรัม ราคา 283.00 บาท</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6VLJcekMgd</t>
+          <t>https://s.shopee.co.th/30lRSHhZGU</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mp3lp4rqcflt1c.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98o-lvaiypl9rum22b.webp</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -1911,46 +1905,46 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>koreadong โคเรียดอง แซลมอนดองซีอิ๊วเกาหลี 1 กระปุก ขนาด 500 กรัม ราคา 283.00 บาท</t>
+          <t>PRO2 *แซลมอนชาคริต* 20 ชิ้น ส่งแช่แข็งฟรี -เนื้อแซลมอน นอร์เวย์ ไร้ก้าง ทานดิบได้- ร้านของคริต ชาคริต แย้มนาม ร้านชาคริต ราคา 3099.00 บาท</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/30lRSHhZGU</t>
+          <t>https://s.shopee.co.th/5q5cpPcaAJ</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98o-lvaiypl9rum22b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-ml5rl1atqqyq13.webp</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>done 2026-06-15 05:50</t>
+          <t>done 2026-06-15 05:51</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PRO2 *แซลมอนชาคริต* 20 ชิ้น ส่งแช่แข็งฟรี -เนื้อแซลมอน นอร์เวย์ ไร้ก้าง ทานดิบได้- ร้านของคริต ชาคริต แย้มนาม ร้านชาคริต ราคา 3099.00 บาท</t>
+          <t>(แพ็ก 12) Muek Groob หมึกกรุบ เส้นบุกปรุงรสหม่าล่า สูตรดั้งเดิม หมึกกรุบซันซุ sunsu ราคา 270.00 บาท</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5q5cpPcaAJ</t>
+          <t>https://s.shopee.co.th/7fXH0qnVjj</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-ml5rl1atqqyq13.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823qs-mp3qgnwmeept30.webp</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -1961,21 +1955,21 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>(แพ็ก 12) Muek Groob หมึกกรุบ เส้นบุกปรุงรสหม่าล่า สูตรดั้งเดิม หมึกกรุบซันซุ sunsu ราคา 270.00 บาท</t>
+          <t>หมูสามชั้นแดดเดียวไร้หนัง สะอาด ปลอดภัย ไม่ใส่สารกันเสีย ไม่ใส่สีผสมอาหาร ทำสดใหม่ทุกวัน ราคา 152.00 บาท</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7fXH0qnVjj</t>
+          <t>https://s.shopee.co.th/1qZU4Lgl3I</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-823qs-mp3qgnwmeept30.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mhshbqn5vy848f.webp</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -1986,46 +1980,46 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>หมูสามชั้นแดดเดียวไร้หนัง สะอาด ปลอดภัย ไม่ใส่สารกันเสีย ไม่ใส่สีผสมอาหาร ทำสดใหม่ทุกวัน ราคา 152.00 บาท</t>
+          <t>ชุด 4 ขวด นมแดรี่โฮมไฮโปรตีน สูตรแลคโตสฟรี ขนาด 300 มล. **จัดส่งเฉพาะในกรุงเทพ** (ไม่มีแถมลังโฟม) ราคา 300.00 บาท</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1qZU4Lgl3I</t>
+          <t>https://s.shopee.co.th/8Kmxo93MVt</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mhshbqn5vy848f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mogz3i52c64t0b.webp</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>done 2026-06-15 05:51</t>
+          <t>done 2026-06-16 06:24</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ชุด 4 ขวด นมแดรี่โฮมไฮโปรตีน สูตรแลคโตสฟรี ขนาด 300 มล. **จัดส่งเฉพาะในกรุงเทพ** (ไม่มีแถมลังโฟม) ราคา 300.00 บาท</t>
+          <t>มันหนึบญี่ปุ่น เบนิฮารุกะ หวานธรรมชาติ ไม่ใส่น้ำตาล ร้านมาซาริ ราคา 272.00 บาท</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8Kmxo93MVt</t>
+          <t>https://s.shopee.co.th/8fPoCyWB2R</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mogz3i52c64t0b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-m70vmyupwyzzda.webp</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2036,21 +2030,21 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>มันหนึบญี่ปุ่น เบนิฮารุกะ หวานธรรมชาติ ไม่ใส่น้ำตาล ร้านมาซาริ ราคา 272.00 บาท</t>
+          <t>🦐 กุ้งแม่น้ำไซส์จัมโป้ 4-7ตัวโล กุ้งตัวใหญ่ๆ 1แพ็คมี3-5ตัว น้ำหนัก1กิโลกรัมน้ำหนักอาจหายนะครับกุ้งสดๆและนำไปแช็ง ราคา 280.00 บาท</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8fPoCyWB2R</t>
+          <t>https://s.shopee.co.th/5Apw2WO73q</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-m70vmyupwyzzda.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mlpbfq1962o574.webp</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2061,21 +2055,21 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>🦐 กุ้งแม่น้ำไซส์จัมโป้ 4-7ตัวโล กุ้งตัวใหญ่ๆ 1แพ็คมี3-5ตัว น้ำหนัก1กิโลกรัมน้ำหนักอาจหายนะครับกุ้งสดๆและนำไปแช็ง ราคา 280.00 บาท</t>
+          <t>เมล็ดเจีย Organic มี อย.คัดพิเศษ เกรดพรีเมี่ยม แบรนด์ไร่พระจันทร์ chia seed 200 400กรัม ราคา 130.00 บาท</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5Apw2WO73q</t>
+          <t>https://s.shopee.co.th/20suGeAdc0</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mlpbfq1962o574.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mkv374joghds15.webp</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2086,21 +2080,21 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>เมล็ดเจีย Organic มี อย.คัดพิเศษ เกรดพรีเมี่ยม แบรนด์ไร่พระจันทร์ chia seed 200 400กรัม ราคา 130.00 บาท</t>
+          <t>ถูกที่สุด Bertolli Extra Virgin Olive Oil เบอร์ทอลลีน้ำมันมะกอกเอ็กซ์ตร้าเวอร์จิ้น ราคา 442.00 บาท</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/20suGeAdc0</t>
+          <t>https://s.shopee.co.th/7fXH0u6NAg</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mkv374joghds15.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-7rbn7-m5xznx46gpavb2.webp</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2111,46 +2105,46 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ถูกที่สุด Bertolli Extra Virgin Olive Oil เบอร์ทอลลีน้ำมันมะกอกเอ็กซ์ตร้าเวอร์จิ้น ราคา 442.00 บาท</t>
+          <t>(แพ็ค 24 ซอง) Muek Groob หมึกกรุบ เส้นบุกปรุงรสหม่าล่า (เลือกรสชาติได้) ราคา 529.00 บาท</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7fXH0u6NAg</t>
+          <t>https://s.shopee.co.th/20ssCZUVx7</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-7rbn7-m5xznx46gpavb2.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mp4md3z4eyvi66.webp</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>done 2026-06-16 06:24</t>
+          <t>done 2026-06-17 06:09</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>(แพ็ค 24 ซอง) Muek Groob หมึกกรุบ เส้นบุกปรุงรสหม่าล่า (เลือกรสชาติได้) ราคา 529.00 บาท</t>
+          <t>ขนมเปี๊ยะไส้ทะลัก ไข่แดงเค็ม 3 ใบ มีให้เลือก 4 รสชาติ ขนาด 450 กรัม WANWANACH ราคา 139.00 บาท</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/20ssCZUVx7</t>
+          <t>https://s.shopee.co.th/8V6O0gAxW4</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mp4md3z4eyvi66.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mmprjgiy639d92.webp</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2161,46 +2155,46 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ขนมเปี๊ยะไส้ทะลัก ไข่แดงเค็ม 3 ใบ มีให้เลือก 4 รสชาติ ขนาด 450 กรัม WANWANACH ราคา 139.00 บาท</t>
+          <t>(6.6) koreadong โคเรียดอง แซลมอนดองซีอิ๊วเกาหลี 4 กระปุก สุดฮิต แถมฟรีน้ำจิ้ม ราคา 1112.00 บาท</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8V6O0gAxW4</t>
+          <t>https://s.shopee.co.th/9AM4nY110F</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mmprjgiy639d92.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mp3lys3nslqk0b.webp</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>done 2026-06-17 06:09</t>
+          <t>done 2026-06-17 06:10</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>(6.6) koreadong โคเรียดอง แซลมอนดองซีอิ๊วเกาหลี 4 กระปุก สุดฮิต แถมฟรีน้ำจิ้ม ราคา 1112.00 บาท</t>
+          <t>Teelek Nougat -นูกัตถุงใหญ่ 18 ชิ้น ราคา 250.00 บาท</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9AM4nY110F</t>
+          <t>https://s.shopee.co.th/4ftfRb84dJ</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mp3lys3nslqk0b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0i-mbrwl55927v730.webp</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2211,21 +2205,21 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Teelek Nougat -นูกัตถุงใหญ่ 18 ชิ้น ราคา 250.00 บาท</t>
+          <t>Country Sourdough Bread ขนมปังซาวโดว์โฮมเมด 100% | SOURDOUGH BREAD | ราคา 182.00 บาท</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4ftfRb84dJ</t>
+          <t>https://s.shopee.co.th/9AM2jit34K</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0i-mbrwl55927v730.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0h-mcpd1y74lysm7e.webp</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2236,46 +2230,46 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Country Sourdough Bread ขนมปังซาวโดว์โฮมเมด 100% | SOURDOUGH BREAD | ราคา 182.00 บาท</t>
+          <t>(มาใหม่)ดูไบคิมบับ ดูไบคุกกี้ชิววี่ เวฟไฟอ่อน10-15วิ ก่อนทาน เพิ่มความฉ่ำ ความยืด ยิ่งอร่อยยิ่งฟิน ตุ๊กกี้ตัวแสบ ราคา 129.00 บาท</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9AM2jit34K</t>
+          <t>https://s.shopee.co.th/W46TihThK</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0h-mcpd1y74lysm7e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mm00dhdvnqbpce.webp</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>done 2026-06-17 06:10</t>
+          <t>done 2026-06-19 06:24</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>(มาใหม่)ดูไบคิมบับ ดูไบคุกกี้ชิววี่ เวฟไฟอ่อน10-15วิ ก่อนทาน เพิ่มความฉ่ำ ความยืด ยิ่งอร่อยยิ่งฟิน ตุ๊กกี้ตัวแสบ ราคา 129.00 บาท</t>
+          <t>นมแพะ Smart Goat 3 ลัง - นมเเพะ ขับถ่ายดี สารอาหารสูง สูตร มัลติวิตามิน &amp; Omega ราคา 2180.00 บาท</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/W46TihThK</t>
+          <t>https://s.shopee.co.th/8ATXc38AC9</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mm00dhdvnqbpce.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasl-maayycy88cayfa.webp</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2286,21 +2280,21 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>นมแพะ Smart Goat 3 ลัง - นมเเพะ ขับถ่ายดี สารอาหารสูง สูตร มัลติวิตามิน &amp; Omega ราคา 2180.00 บาท</t>
+          <t>สลิดติดปาก ปลาสลิดแดดเดียว 5-6 ตัว/โล | ปลาสลิดไข่บางบ่อ ตัวโต สด สะอาด เนื้อแน่นหอมมัน ราคา 469.00 บาท</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8ATXc38AC9</t>
+          <t>https://s.shopee.co.th/4ftfRc0nMj</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasl-maayycy88cayfa.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mgvmi6civ40e0a.webp</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2311,21 +2305,21 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>สลิดติดปาก ปลาสลิดแดดเดียว 5-6 ตัว/โล | ปลาสลิดไข่บางบ่อ ตัวโต สด สะอาด เนื้อแน่นหอมมัน ราคา 469.00 บาท</t>
+          <t>(ซื้อ 1 แถม 2)Matcha Japan ผงมัทฉะ ออร์แกนิค (Organic Matcha Powder) ขนาด 300g ขนาด ไม่ผสมแป้ง ไม่ผสมน้ำตาล ทานง่ายไม่ขม ราคา 351.00 บาท</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4ftfRc0nMj</t>
+          <t>https://s.shopee.co.th/1BJnGu1X1D</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mgvmi6civ40e0a.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-7ren5-mdu2gpkdaiop19.webp</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2336,21 +2330,21 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>(ซื้อ 1 แถม 2)Matcha Japan ผงมัทฉะ ออร์แกนิค (Organic Matcha Powder) ขนาด 300g ขนาด ไม่ผสมแป้ง ไม่ผสมน้ำตาล ทานง่ายไม่ขม ราคา 351.00 บาท</t>
+          <t>น้ำพริกปูม้า(เจ๊เล็กน้ำพริกปูม้า),ฮาลาลฟู๊ด,มี6สูตร มันปูม้า/ไข่ปูม้า/เนื้อปูม้า/สไปซี่/ไข่เผ็ดน้อย ราคา 147.00 บาท</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1BJnGu1X1D</t>
+          <t>https://s.shopee.co.th/80A7PfAPBU</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-7ren5-mdu2gpkdaiop19.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasl-m5phtrsv3qy25c.webp</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2361,46 +2355,46 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>น้ำพริกปูม้า(เจ๊เล็กน้ำพริกปูม้า),ฮาลาลฟู๊ด,มี6สูตร มันปูม้า/ไข่ปูม้า/เนื้อปูม้า/สไปซี่/ไข่เผ็ดน้อย ราคา 147.00 บาท</t>
+          <t>ICHITAN อิชิตัน น้ำด่าง ผสมวิตามินบีรวม ขนาดใหญ่ 550 ml. 1 ลัง (24 ขวด) รวมจัดส่ง ราคา 480.00 บาท</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/80A7PfAPBU</t>
+          <t>https://s.shopee.co.th/9AM4ngSAXx</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasl-m5phtrsv3qy25c.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-m3byqpp14oa0c1.webp</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>done 2026-06-19 06:24</t>
+          <t>done 2026-06-20 05:37</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ICHITAN อิชิตัน น้ำด่าง ผสมวิตามินบีรวม ขนาดใหญ่ 550 ml. 1 ลัง (24 ขวด) รวมจัดส่ง ราคา 480.00 บาท</t>
+          <t>พร้อมส่งในไทย Marukyu​ Koyamaen​ ผงมัทฉะ​ มารุคิวของแท้จากญี่ปุ่น​ Matcha​ มัทฉะยี่ห้อดังจากอูจิ ราคา 760.00 บาท</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9AM4ngSAXx</t>
+          <t>https://s.shopee.co.th/6VLJclpvLq</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-m3byqpp14oa0c1.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mn5j25gwgmx2ed.webp</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2411,46 +2405,46 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>พร้อมส่งในไทย Marukyu​ Koyamaen​ ผงมัทฉะ​ มารุคิวของแท้จากญี่ปุ่น​ Matcha​ มัทฉะยี่ห้อดังจากอูจิ ราคา 760.00 บาท</t>
+          <t>Kanbayashi Shunsho.มัทฉะ Matcha ZUIHO/ชาเขียว/ชาเขียวมัทฉะ/ผงมัทฉะ/ลูกร่อนผงมัทฉะ/มัทฉะโทนถั่ว ราคา 1048.00 บาท</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6VLJclpvLq</t>
+          <t>https://s.shopee.co.th/4qD5dYKnKI</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mn5j25gwgmx2ed.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasi-m76lcjji3bcfb4.webp</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>done 2026-06-20 05:37</t>
+          <t>done 2026-06-20 05:38</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Kanbayashi Shunsho.มัทฉะ Matcha ZUIHO/ชาเขียว/ชาเขียวมัทฉะ/ผงมัทฉะ/ลูกร่อนผงมัทฉะ/มัทฉะโทนถั่ว ราคา 1048.00 บาท</t>
+          <t>หมูเเดดเดียว 500 กรัม เจ๊ติ๋ม ตลาด อ.ต.ก.เจ้าเก่า (30ปี) "สูตรอร่อยไม่มีใครเหมือน" ราคา 194.00 บาท</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4qD5dYKnKI</t>
+          <t>https://s.shopee.co.th/8fPoCzE2Lb</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasi-m76lcjji3bcfb4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/3f7c3f4a61b0bef5b99b1041e212dfe4.webp</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -2461,21 +2455,21 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>หมูเเดดเดียว 500 กรัม เจ๊ติ๋ม ตลาด อ.ต.ก.เจ้าเก่า (30ปี) "สูตรอร่อยไม่มีใครเหมือน" ราคา 194.00 บาท</t>
+          <t>ตราฉัตร 5 กิโล ข้าวหอมมะลิใหม่ ข้าวหอมมะลิแท้ ตราฉัตร 5kg. (หอม นุ่ม ตลอดปี) ข้าวหอมผสม ข้าวขาว หุงอร่อย หุงขึ้นหม้อ ราคา 145.00 บาท</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8fPoCzE2Lb</t>
+          <t>https://s.shopee.co.th/4AxOqdHAb1</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/3f7c3f4a61b0bef5b99b1041e212dfe4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-8260m-mkdsz738rxtu0a.webp</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -2486,46 +2480,46 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ตราฉัตร 5 กิโล ข้าวหอมมะลิใหม่ ข้าวหอมมะลิแท้ ตราฉัตร 5kg. (หอม นุ่ม ตลอดปี) ข้าวหอมผสม ข้าวขาว หุงอร่อย หุงขึ้นหม้อ ราคา 145.00 บาท</t>
+          <t>1แถม1ขนมโมจิมีนม่วงญี่ปุ่น หอม หวาน มัน ราคา 98.00 บาท</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4AxOqdHAb1</t>
+          <t>https://s.shopee.co.th/7KuQcRjWpZ</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-8260m-mkdsz738rxtu0a.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mfun2mvlmk25c6.webp</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>done 2026-06-20 05:38</t>
+          <t>done 2026-06-21 05:49</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>1แถม1ขนมโมจิมีนม่วงญี่ปุ่น หอม หวาน มัน ราคา 98.00 บาท</t>
+          <t>Nao Matcha นาโอะ มัทฉะแท้ 100% เกรดพรีเมียมจากนิชิโอะ ญี่ปุ่น หอมนัว Nutty ไม่ขม ไม่ฝาด ขนาด 40g ราคา 290.00 บาท</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7KuQcRjWpZ</t>
+          <t>https://s.shopee.co.th/5VSmQuoqES</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mfun2mvlmk25c6.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mn9qqsw8mtqab0.webp</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -2536,21 +2530,21 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Nao Matcha นาโอะ มัทฉะแท้ 100% เกรดพรีเมียมจากนิชิโอะ ญี่ปุ่น หอมนัว Nutty ไม่ขม ไม่ฝาด ขนาด 40g ราคา 290.00 บาท</t>
+          <t>Esan phasuab น้ำปลาร้าอีสานพาสวบ 3ขวด (ขวดละ350มล) หอมกลิ่นปลาร้าแท้ สูตรแซบนัว สำหรับส้มตำและอาหาร ราคา 180.00 บาท</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5VSmQuoqES</t>
+          <t>https://s.shopee.co.th/3g18FWNAGN</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mn9qqsw8mtqab0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qukz-lhj88jai5qmrb3.webp</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -2561,21 +2555,21 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Esan phasuab น้ำปลาร้าอีสานพาสวบ 3ขวด (ขวดละ350มล) หอมกลิ่นปลาร้าแท้ สูตรแซบนัว สำหรับส้มตำและอาหาร ราคา 180.00 บาท</t>
+          <t>นมเปรี้ยว ดัชมิลล์ ขนาด 180 ml เซต 5 แพ็ค มี 5 รสชาติ คละรสให้อย่างละ 1แพ็ค (4 กล่อง/แพ็ค) ราคา 250.00 บาท</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3g18FWNAGN</t>
+          <t>https://s.shopee.co.th/902ebaZJA4</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7qukz-lhj88jai5qmrb3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m0hc9m3k5g3e37.webp</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -2586,21 +2580,21 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>นมเปรี้ยว ดัชมิลล์ ขนาด 180 ml เซต 5 แพ็ค มี 5 รสชาติ คละรสให้อย่างละ 1แพ็ค (4 กล่อง/แพ็ค) ราคา 250.00 บาท</t>
+          <t>แคบหมูไร้มัน แคปหมูไร้มัน 1kg. 500g. ราคา 219.00 บาท</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/902ebaZJA4</t>
+          <t>https://s.shopee.co.th/30lRSLg5c1</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m0hc9m3k5g3e37.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-macyz9o9j8fof8.webp</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -2611,71 +2605,71 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>แคบหมูไร้มัน แคปหมูไร้มัน 1kg. 500g. ราคา 219.00 บาท</t>
+          <t>กาแฟดำเพื่อสุขภาพ ไม่มีน้ำตาล คั่วสด บดละเอียด ผงสกัดกาแฟละลายน้ำร้อนทันที พร้อมดื่ม Healthy Black Coffee | ร้านกาแฟ 89 ราคา 99.00 บาท</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/30lRSLg5c1</t>
+          <t>https://s.shopee.co.th/6VLHYpGKZE</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-macyz9o9j8fof8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98r-ly99vph2c04pdc.webp</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>done 2026-06-21 05:49</t>
+          <t>done 2026-06-22 05:48</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>กาแฟดำเพื่อสุขภาพ ไม่มีน้ำตาล คั่วสด บดละเอียด ผงสกัดกาแฟละลายน้ำร้อนทันที พร้อมดื่ม Healthy Black Coffee | ร้านกาแฟ 89 ราคา 99.00 บาท</t>
+          <t>ทุเรียนจันทบุรีเนื้อพรีเมียม ยอดขายเยอะที่สุดทุเรียนหมอนทอง คัดเนื้อเทพไม่เน้นทรง เนื้อเหลือง เนื้อตลาดที่คนไทยกิน ราคา 621.00 บาท</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6VLHYpGKZE</t>
+          <t>https://s.shopee.co.th/2LVibAwjEv</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98r-ly99vph2c04pdc.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rask-mabmx8hshx6278.webp</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>done 2026-06-22 05:48</t>
+          <t>done 2026-06-22 05:49</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ทุเรียนจันทบุรีเนื้อพรีเมียม ยอดขายเยอะที่สุดทุเรียนหมอนทอง คัดเนื้อเทพไม่เน้นทรง เนื้อเหลือง เนื้อตลาดที่คนไทยกิน ราคา 621.00 บาท</t>
+          <t>พริกกากหมู เคี้ยวเพลินๆ(รสต้มยำ) ราคา 150.00 บาท</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2LVibAwjEv</t>
+          <t>https://s.shopee.co.th/5Apw2C68Zb</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rask-mabmx8hshx6278.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mgl58k2i07ii90.webp</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -2686,21 +2680,21 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>พริกกากหมู เคี้ยวเพลินๆ(รสต้มยำ) ราคา 150.00 บาท</t>
+          <t>ทุเรียนหมอนทอง คัดพิเศษ กล่องใหญ่ 3.5 กก. ราคา 3700.00 บาท</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5Apw2C68Zb</t>
+          <t>https://s.shopee.co.th/8pjEP0uUQS</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mgl58k2i07ii90.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/f8fb32659a3650ce0dcc468f645e65be.webp</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -2711,21 +2705,21 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ทุเรียนหมอนทอง คัดพิเศษ กล่องใหญ่ 3.5 กก. ราคา 3700.00 บาท</t>
+          <t>[✅โค้ดส่งฟรี+🎫โค้ดคุุ้ม] น้ำปลาร้าปรุงสุก ตราไมค์ 6 ขวด ขนาด 350 ml. (แซ่บไมค์) น้ำปลาร้า ปรุงสุก สูตรแซ่บทุกเมนู ราคา 245.00 บาท</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8pjEP0uUQS</t>
+          <t>https://s.shopee.co.th/60P31jKZ0f</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/f8fb32659a3650ce0dcc468f645e65be.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-mab0imamdy4f32.webp</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -2736,71 +2730,71 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>[✅โค้ดส่งฟรี+🎫โค้ดคุุ้ม] น้ำปลาร้าปรุงสุก ตราไมค์ 6 ขวด ขนาด 350 ml. (แซ่บไมค์) น้ำปลาร้า ปรุงสุก สูตรแซ่บทุกเมนู ราคา 245.00 บาท</t>
+          <t>แอปเปิ้ลแช่แข็งแห้งกรอบพรีเมี่ยมชิ้นไม่มีสารเติมแต่งขนมขบเคี้ยวผลไม้แห้งสําหรับผู้ใหญ่ของว่างเพื่อสุขภาพแบบสบาย ๆ ราคา 112.00 บาท</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/60P31jKZ0f</t>
+          <t>https://s.shopee.co.th/6AiTE9uySD</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-mab0imamdy4f32.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-mn06agdyktfl55.webp</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>done 2026-06-22 05:49</t>
+          <t>done 2026-06-23 06:05</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>แอปเปิ้ลแช่แข็งแห้งกรอบพรีเมี่ยมชิ้นไม่มีสารเติมแต่งขนมขบเคี้ยวผลไม้แห้งสําหรับผู้ใหญ่ของว่างเพื่อสุขภาพแบบสบาย ๆ ราคา 112.00 บาท</t>
+          <t>น้ำพริกแห้งปลาสลิดโรยข้าว รสผัดพริกขิง รสสมุนไพร รสน้ำพริกนรก แบบซอง ขนาด 100 กรัม 3 รสชาติ 1 ซอง Zalidpordeekum ราคา 155.00 บาท</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6AiTE9uySD</t>
+          <t>https://s.shopee.co.th/7VDqoXVW0v</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-mn06agdyktfl55.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m863k6w28arga0.webp</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>done 2026-06-23 06:05</t>
+          <t>done 2026-06-23 06:06</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>น้ำพริกแห้งปลาสลิดโรยข้าว รสผัดพริกขิง รสสมุนไพร รสน้ำพริกนรก แบบซอง ขนาด 100 กรัม 3 รสชาติ 1 ซอง Zalidpordeekum ราคา 155.00 บาท</t>
+          <t>กรุงเทพปริมณฑลมีส่งด่วนยอดขายมากที่สุด รีวิวมากที่สุด ทุเรียนหมอนทองจันทบุรีแกะเนื้อ ราคา 542.00 บาท</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7VDqoXVW0v</t>
+          <t>https://s.shopee.co.th/9fILOohMBk</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m863k6w28arga0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/4fb7d47caa67d61241a2af680a4ad3a6.webp</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -2811,21 +2805,21 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>กรุงเทพปริมณฑลมีส่งด่วนยอดขายมากที่สุด รีวิวมากที่สุด ทุเรียนหมอนทองจันทบุรีแกะเนื้อ ราคา 542.00 บาท</t>
+          <t>เนสกาแฟ​ nescafe กาแฟ​สำเร็จ​รูป ราคา 173.00 บาท</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fILOohMBk</t>
+          <t>https://s.shopee.co.th/6VLJckD4gB</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/4fb7d47caa67d61241a2af680a4ad3a6.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mjrwzih0tts540.webp</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -2836,21 +2830,21 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>เนสกาแฟ​ nescafe กาแฟ​สำเร็จ​รูป ราคา 173.00 บาท</t>
+          <t>เนยถั่วรวม Chocolate Nuts Butter รสช็อคโกแลต ขนาด 220 g. | Paweenee’s ราคา 175.00 บาท</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6VLJckD4gB</t>
+          <t>https://s.shopee.co.th/20suGfEdLr</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mjrwzih0tts540.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0j-mdoxiej3ykficb.webp</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -2861,46 +2855,46 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>เนยถั่วรวม Chocolate Nuts Butter รสช็อคโกแลต ขนาด 220 g. | Paweenee’s ราคา 175.00 บาท</t>
+          <t>อึ่งไข่ฝนแรก ❗️พร้อมส่ง อึ่งไข่แช่แข็ง 📍อึ่งไข่ฝนแรกล็อตสุดท้ายของปีนี้ ราคา 850.00 บาท</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/20suGfEdLr</t>
+          <t>https://s.shopee.co.th/1VwdfVn8Ft</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0j-mdoxiej3ykficb.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m8x3w0uh4ci73e.webp</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>done 2026-06-23 06:06</t>
+          <t>done 2026-06-24 05:51</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>อึ่งไข่ฝนแรก ❗️พร้อมส่ง อึ่งไข่แช่แข็ง 📍อึ่งไข่ฝนแรกล็อตสุดท้ายของปีนี้ ราคา 850.00 บาท</t>
+          <t>หมูแดดเดียวพรีเมียม อบลมร้อน สะอาด ไร้ฝุ่น ไร้แมลง เนื้อนุ่ม ฉ่ำ ทอดง่าย ราคา 149.00 บาท</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1VwdfVn8Ft</t>
+          <t>https://s.shopee.co.th/2g8YznZTBU</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m8x3w0uh4ci73e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mm8rnpzzshs429.webp</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -2911,21 +2905,21 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>หมูแดดเดียวพรีเมียม อบลมร้อน สะอาด ไร้ฝุ่น ไร้แมลง เนื้อนุ่ม ฉ่ำ ทอดง่าย ราคา 149.00 บาท</t>
+          <t>ชามะระขี้นก ตราทองหลวง ☘️❇️ ของเเท้ พร้อมส่ง📌 ราคา 80.00 บาท</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2g8YznZTBU</t>
+          <t>https://s.shopee.co.th/9zvBnPVuA0</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mm8rnpzzshs429.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m3hccjp1scl7d9.webp</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -2936,21 +2930,21 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ชามะระขี้นก ตราทองหลวง ☘️❇️ ของเเท้ พร้อมส่ง📌 ราคา 80.00 บาท</t>
+          <t>[พร้อมส่งในไทย]Marukyu Koyamaen Matcha มัทฉะมารุคิวโคยามะเอ็น สาหร่ายผู้ดี อูมามิ เกรดพิธีการญี่ปุ่น ราคา 1118.00 บาท</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9zvBnPVuA0</t>
+          <t>https://s.shopee.co.th/902ebFHsE7</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m3hccjp1scl7d9.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m91el64l52bt32.webp</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -2961,71 +2955,71 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>[พร้อมส่งในไทย]Marukyu Koyamaen Matcha มัทฉะมารุคิวโคยามะเอ็น สาหร่ายผู้ดี อูมามิ เกรดพิธีการญี่ปุ่น ราคา 1118.00 บาท</t>
+          <t>น้ำพริกหมูกระจกมะเดี่ยว วับวาว รสต้มยำ ชิ้นใหญ่ เต็มคำ แซ่บ เปรี้ยวเผ็ดสะใจ มี2ขนาด 100g./400g. ราคา 365.00 บาท</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/902ebFHsE7</t>
+          <t>https://s.shopee.co.th/20suGMieQS</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m91el64l52bt32.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mnmij2prwhl2a7.webp</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>done 2026-06-24 05:51</t>
+          <t>done 2026-06-24 05:52</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>น้ำพริกหมูกระจกมะเดี่ยว วับวาว รสต้มยำ ชิ้นใหญ่ เต็มคำ แซ่บ เปรี้ยวเผ็ดสะใจ มี2ขนาด 100g./400g. ราคา 365.00 บาท</t>
+          <t>น้ำจิ้มปิ้งย่าง สูตรพี่ฟร้องซ์ **ไม่ใส่ผักชี** กระทะร้อน อร่อยมาก ถึงเครื่อง เข้มข้น ครบรส ราคา 89.00 บาท</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/20suGMieQS</t>
+          <t>https://s.shopee.co.th/9fILOSX406</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mnmij2prwhl2a7.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mp66zmbl7xtt82.webp</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>done 2026-06-24 05:52</t>
+          <t>done 2026-06-25 05:51</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>น้ำจิ้มปิ้งย่าง สูตรพี่ฟร้องซ์ **ไม่ใส่ผักชี** กระทะร้อน อร่อยมาก ถึงเครื่อง เข้มข้น ครบรส ราคา 89.00 บาท</t>
+          <t>น้ำมันปาล์ม เกสร ราคาพิเศษ 3 ขวด ราคา 220.00 บาท</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fILOSX406</t>
+          <t>https://s.shopee.co.th/3LOHqsGZzL</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mp66zmbl7xtt82.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mmtjwuvjtxxf59.webp</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -3036,21 +3030,21 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>น้ำมันปาล์ม เกสร ราคาพิเศษ 3 ขวด ราคา 220.00 บาท</t>
+          <t>คุกกี้ไส้ทะลัก แบบ 6 ชิ้น 10 ชิ้น กระปุกเดี่ยว (เลือกได้ 3 ไส้ ช็อกโกแลต, ไวท์ช็อก, มัทฉะ) ราคา 120.00 บาท</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3LOHqsGZzL</t>
+          <t>https://s.shopee.co.th/60P324DO3F</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mmtjwuvjtxxf59.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mf0sw2zx81sdb8.webp</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -3061,46 +3055,46 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>คุกกี้ไส้ทะลัก แบบ 6 ชิ้น 10 ชิ้น กระปุกเดี่ยว (เลือกได้ 3 ไส้ ช็อกโกแลต, ไวท์ช็อก, มัทฉะ) ราคา 120.00 บาท</t>
+          <t>Benefruit มะพร้าวอบแห้ง🥥 มะพร้าวกรอบ เนื้อแน่นกรึบ หวานน้อย สูตรน้ำตาลต่ำ (Dried Coconut) ราคา 195.00 บาท</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/60P324DO3F</t>
+          <t>https://s.shopee.co.th/8fPm8nVF0k</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mf0sw2zx81sdb8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mg3ydny6nkzwa4.webp</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>done 2026-06-25 05:51</t>
+          <t>done 2026-06-25 05:52</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Benefruit มะพร้าวอบแห้ง🥥 มะพร้าวกรอบ เนื้อแน่นกรึบ หวานน้อย สูตรน้ำตาลต่ำ (Dried Coconut) ราคา 195.00 บาท</t>
+          <t>น้ำมันมรกต 1 ลิตร ยกลัง 12 ขวด สินค้าส่งตรงจากโรงงาน (1 คำสั่งซื้อ 1 ลัง) ต้องการมากกว่า 1 ให้แยกคำสั่งซื้อ ราคา 822.00 บาท</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8fPm8nVF0k</t>
+          <t>https://s.shopee.co.th/AKY2BxEinW</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mg3ydny6nkzwa4.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98u-lnfj2bxeyxioc3.webp</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -3111,46 +3105,46 @@
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>น้ำมันมรกต 1 ลิตร ยกลัง 12 ขวด สินค้าส่งตรงจากโรงงาน (1 คำสั่งซื้อ 1 ลัง) ต้องการมากกว่า 1 ให้แยกคำสั่งซื้อ ราคา 822.00 บาท</t>
+          <t>[จัดให้ 2 กระปุก]🌶️น้ำพริกไข่มันกุ้ง+น้ำพริกไข่ปูมัน รสชาติดีแซ่บนัว เผ็ดกำลังดีกินกับอะไรก็อร่อย ราคา 199.00 บาท</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AKY2BxEinW</t>
+          <t>https://s.shopee.co.th/5L9MEmdTGN</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98u-lnfj2bxeyxioc3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98z-lof5ug62n1lrb6.webp</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>done 2026-06-25 05:52</t>
+          <t>done 2026-06-26 06:02</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>[จัดให้ 2 กระปุก]🌶️น้ำพริกไข่มันกุ้ง+น้ำพริกไข่ปูมัน รสชาติดีแซ่บนัว เผ็ดกำลังดีกินกับอะไรก็อร่อย ราคา 199.00 บาท</t>
+          <t>พริกกากหมู สูตรโบราณดั้งเดิม ราคา 150.00 บาท</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5L9MEmdTGN</t>
+          <t>https://s.shopee.co.th/LkgHbCNxF</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98z-lof5ug62n1lrb6.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mgl5dbuy21vu55.webp</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -3161,21 +3155,21 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>พริกกากหมู สูตรโบราณดั้งเดิม ราคา 150.00 บาท</t>
+          <t>น้ำพริกแซลมอนไข่เค็มคลีน ไม่มัน ไม่ใส่ผงชูรส ไม่ใส่สารกันเสีย ขนาด 150 กรัม ราคา 150.00 บาท</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/LkgHbCNxF</t>
+          <t>https://s.shopee.co.th/7KuOYNPsuy</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mgl5dbuy21vu55.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mkc4ypl093wg43.webp</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -3186,46 +3180,46 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>น้ำพริกแซลมอนไข่เค็มคลีน ไม่มัน ไม่ใส่ผงชูรส ไม่ใส่สารกันเสีย ขนาด 150 กรัม ราคา 150.00 บาท</t>
+          <t>สเต็กเนื้อโคขุนพริกไทยดำ(140-150กรัม/ชิ้น)(10ชิ้น)มีทั้งแบบหมักและยังไม่หมัก ราคา 650.00 บาท</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7KuOYNPsuy</t>
+          <t>https://s.shopee.co.th/5q5alcwc11</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mkc4ypl093wg43.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-23020-776z5w1itknved.webp</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>done 2026-06-26 06:02</t>
+          <t>done 2026-06-26 06:03</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>สเต็กเนื้อโคขุนพริกไทยดำ(140-150กรัม/ชิ้น)(10ชิ้น)มีทั้งแบบหมักและยังไม่หมัก ราคา 650.00 บาท</t>
+          <t>🚚โรงงาน🚚สับปะรดภูแลอบแห้งมินิมอล 齋·حلال สูตรธรรมชาติ ขนาด 100และ500 กรัม สับปะรด สับปะรดอบแห้ง ราคา 150.00 บาท</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5q5alcwc11</t>
+          <t>https://s.shopee.co.th/2LVkfLPdSv</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-23020-776z5w1itknved.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/f07437515d60d68bea2d8cd474eb1eee.webp</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -3236,46 +3230,46 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>🚚โรงงาน🚚สับปะรดภูแลอบแห้งมินิมอล 齋·حلال สูตรธรรมชาติ ขนาด 100และ500 กรัม สับปะรด สับปะรดอบแห้ง ราคา 150.00 บาท</t>
+          <t>ถั่ว 9 เซียน ธัญพืชรวม อบกรุบกรอบ รสดั้งเดิม ออแกนิค ไม่น้ำมัน ไม่เนย VIP Mixed nuts ราคา 199.00 บาท</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2LVkfLPdSv</t>
+          <t>https://s.shopee.co.th/3qKYRjSfM7</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/f07437515d60d68bea2d8cd474eb1eee.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasb-m0pmsf4ero482f.webp</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>done 2026-06-26 06:03</t>
+          <t>done 2026-06-27 05:49</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ถั่ว 9 เซียน ธัญพืชรวม อบกรุบกรอบ รสดั้งเดิม ออแกนิค ไม่น้ำมัน ไม่เนย VIP Mixed nuts ราคา 199.00 บาท</t>
+          <t>ผลไม้อบแห้งพรีเมียม: ลูกเกดและเบอร์รี่ (ลูกเกดเหลือง, ลูกเกดดำ, แครนเบอร์รี่, สตรอว์เบอร์รี่ ราคา 135.00 บาท</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qKYRjSfM7</t>
+          <t>https://s.shopee.co.th/8Kmxo5EbPm</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasb-m0pmsf4ero482f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m0zk8bm0ldm0ab.webp</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -3286,21 +3280,21 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ผลไม้อบแห้งพรีเมียม: ลูกเกดและเบอร์รี่ (ลูกเกดเหลือง, ลูกเกดดำ, แครนเบอร์รี่, สตรอว์เบอร์รี่ ราคา 135.00 บาท</t>
+          <t>ขายดี🔥 Benefruit ส้มอบแห้ง🍊ส้มหนึบ กลีบส้ม ไร้เม็ด ผลไม้อบแห้งเกรดส่งออก สูตรน้ำตาลต่ำ (Dried Orange Low Sugar) ราคา 95.00 บาท</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8Kmxo5EbPm</t>
+          <t>https://s.shopee.co.th/9zvBn7ZKHf</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m0zk8bm0ldm0ab.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m6tjad8k1fxc38.webp</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -3311,46 +3305,46 @@
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ขายดี🔥 Benefruit ส้มอบแห้ง🍊ส้มหนึบ กลีบส้ม ไร้เม็ด ผลไม้อบแห้งเกรดส่งออก สูตรน้ำตาลต่ำ (Dried Orange Low Sugar) ราคา 95.00 บาท</t>
+          <t>น้ำพริกน้ำย้อย ตรายาหยี (สูตรเมืองแพร่ดั้งเดิม) 👉 รสหอมกระเทียม BY ทอดไท/หมวยมาลี ราคา 97.00 บาท</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9zvBn7ZKHf</t>
+          <t>https://s.shopee.co.th/3qKYRqd2O6</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m6tjad8k1fxc38.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m26a2qtnb0f59d.webp</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>done 2026-06-27 05:49</t>
+          <t>done 2026-06-27 05:50</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>น้ำพริกน้ำย้อย ตรายาหยี (สูตรเมืองแพร่ดั้งเดิม) 👉 รสหอมกระเทียม BY ทอดไท/หมวยมาลี ราคา 97.00 บาท</t>
+          <t>[มี อ.ย.‼] ซอสผัดกะเพรา สูตรเข้มข้น ตราใบเพรา ขนาด 500 ml. (ส่งของทุกวัน) ราคา 119.00 บาท</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qKYRqd2O6</t>
+          <t>https://s.shopee.co.th/6AiTE2tGTE</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m26a2qtnb0f59d.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-lv5y3stoku1p7e.webp</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -3361,46 +3355,46 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>[มี อ.ย.‼] ซอสผัดกะเพรา สูตรเข้มข้น ตราใบเพรา ขนาด 500 ml. (ส่งของทุกวัน) ราคา 119.00 บาท</t>
+          <t>หมูสามชั้นทอดน้ำปลา ตรา ทอดไท 🔥พร้อมทาน 👉 100/200 ก. ราคา 109.00 บาท</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6AiTE2tGTE</t>
+          <t>https://s.shopee.co.th/60P0xuwNip</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-lv5y3stoku1p7e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98t-lr10flflo1x932.webp</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>done 2026-06-27 05:50</t>
+          <t>done 2026-06-28 05:43</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>หมูสามชั้นทอดน้ำปลา ตรา ทอดไท 🔥พร้อมทาน 👉 100/200 ก. ราคา 109.00 บาท</t>
+          <t>มัทฉะ Kanbayashi Shunsho Koicha Zuihou ซุยโหว Uji matcha powder 20g/40g【ส่งตรงจากญี่ปุ่น】 ราคา 1854.00 บาท</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/60P0xuwNip</t>
+          <t>https://s.shopee.co.th/7fXH0ll3wH</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98t-lr10flflo1x932.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mj7uce60pq1137.webp</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -3411,21 +3405,21 @@
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>มัทฉะ Kanbayashi Shunsho Koicha Zuihou ซุยโหว Uji matcha powder 20g/40g【ส่งตรงจากญี่ปุ่น】 ราคา 1854.00 บาท</t>
+          <t>สตรอว์เบอร์รี่ คลุกพริกเกลือ จี๊ดจ๊าดชื่นใจ ลูกใหญ่ เนื้อนุ่มหนึบ ไม่แข็ง ราคา 189.00 บาท</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7fXH0ll3wH</t>
+          <t>https://s.shopee.co.th/2BCKSwb0pY</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mj7uce60pq1137.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lp8wi9tav0ji70.webp</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -3436,21 +3430,21 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>สตรอว์เบอร์รี่ คลุกพริกเกลือ จี๊ดจ๊าดชื่นใจ ลูกใหญ่ เนื้อนุ่มหนึบ ไม่แข็ง ราคา 189.00 บาท</t>
+          <t>โรตีสายไหมทุเรียนแม่ระย้า โรตีสายไหมอยุธยา พร้อมส่งด่วนทั่วประเทศ ซีลแป้งถุงสูญญากาศ ราคา 119.00 บาท</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2BCKSwb0pY</t>
+          <t>https://s.shopee.co.th/30lPOOlK3t</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lp8wi9tav0ji70.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mjebq9kba60z58.webp</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -3461,71 +3455,71 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>โรตีสายไหมทุเรียนแม่ระย้า โรตีสายไหมอยุธยา พร้อมส่งด่วนทั่วประเทศ ซีลแป้งถุงสูญญากาศ ราคา 119.00 บาท</t>
+          <t>แพ็คเกจใหม่ น้ำพริกหมูกระจก รสต้มยำ ขนาด 500 กรัม ราคา 270.00 บาท</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/30lPOOlK3t</t>
+          <t>https://s.shopee.co.th/AUrSO2T1U0</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mjebq9kba60z58.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-ml68c61fho8w10.webp</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>done 2026-06-28 05:43</t>
+          <t>done 2026-06-28 05:44</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>แพ็คเกจใหม่ น้ำพริกหมูกระจก รสต้มยำ ขนาด 500 กรัม ราคา 270.00 บาท</t>
+          <t>หมูกรอบ เงินล้าน เนื้อเยอะ มันน้อย เนื้อแน่น หนังกรอบ กรอบนอกนุ่มใน พร้อมน้ำจิ้ม ขนาด 500ก./ 1,000ก. ราคา 290.00 บาท</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AUrSO2T1U0</t>
+          <t>https://s.shopee.co.th/2qS1FtJTov</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-ml68c61fho8w10.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rask-m76elywra3an63.webp</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>done 2026-06-28 05:44</t>
+          <t>done 2026-06-29 05:43</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>หมูกรอบ เงินล้าน เนื้อเยอะ มันน้อย เนื้อแน่น หนังกรอบ กรอบนอกนุ่มใน พร้อมน้ำจิ้ม ขนาด 500ก./ 1,000ก. ราคา 290.00 บาท</t>
+          <t>แพ็คเกจใหม่ รวม น้ำพริกหมูกระจก ขนาด 500 กรัม ราคา 270.00 บาท</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qS1FtJTov</t>
+          <t>https://s.shopee.co.th/3g18FVFWd9</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rask-m76elywra3an63.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-ml680l0flgxt0f.webp</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -3536,21 +3530,21 @@
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>แพ็คเกจใหม่ รวม น้ำพริกหมูกระจก ขนาด 500 กรัม ราคา 270.00 บาท</t>
+          <t>ผงมัทฉะนิชิโอะ เกรดพรีเมี่ยม Noko 100 กรัม | Premium Grade Nishio Matcha Powder ราคา 600.00 บาท</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3g18FVFWd9</t>
+          <t>https://s.shopee.co.th/3g18FVwHjP</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-ml680l0flgxt0f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mk3h45kcwrnpc8.webp</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -3561,21 +3555,21 @@
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>ผงมัทฉะนิชิโอะ เกรดพรีเมี่ยม Noko 100 กรัม | Premium Grade Nishio Matcha Powder ราคา 600.00 บาท</t>
+          <t>ส่งด่วน กรุงเทพ/ตจว.❤️ทุเรียนป่าละอู 1โลเนื้อล้วน🧡เนื้อละมุน หวานมัน ปีละครั้ง ต้องลอง🍉 ส่งด่วนทุกวัน ทั่วประเทศ ราคา 849.00 บาท</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3g18FVwHjP</t>
+          <t>https://s.shopee.co.th/8ATXbpvKoM</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mk3h45kcwrnpc8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0n-md1gusdgvf2880.webp</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -3586,21 +3580,21 @@
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>ส่งด่วน กรุงเทพ/ตจว.❤️ทุเรียนป่าละอู 1โลเนื้อล้วน🧡เนื้อละมุน หวานมัน ปีละครั้ง ต้องลอง🍉 ส่งด่วนทุกวัน ทั่วประเทศ ราคา 849.00 บาท</t>
+          <t>อุดมสุข นรกแซลมอน 100 กรัม น้ำพริกคลีน น้ำพริกคีโต น้ำพริกเพื่อสุขภาพ อาหารคลีน อาหารคีโต ราคา 159.00 บาท</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8ATXbpvKoM</t>
+          <t>https://s.shopee.co.th/17pspiEJT</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0n-md1gusdgvf2880.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mk5i8ralf11k25.webp</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -3611,71 +3605,71 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>อุดมสุข นรกแซลมอน 100 กรัม น้ำพริกคลีน น้ำพริกคีโต น้ำพริกเพื่อสุขภาพ อาหารคลีน อาหารคีโต ราคา 159.00 บาท</t>
+          <t>ชาเขียว 100% เพียวมัทฉะ ชาเขียว พรีเมี่ยม matcha powder from japan 0 สารเติมแต่ง 1 กระป๋อง 300g ราคา 355.00 บาท</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/17pspiEJT</t>
+          <t>https://s.shopee.co.th/4AxOqM1Q5R</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mk5i8ralf11k25.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mhivoyzzzqird0.webp</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>done 2026-06-29 05:43</t>
+          <t>done 2026-06-30 05:40</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ชาเขียว 100% เพียวมัทฉะ ชาเขียว พรีเมี่ยม matcha powder from japan 0 สารเติมแต่ง 1 กระป๋อง 300g ราคา 355.00 บาท</t>
+          <t>น้ำพริกผัดหมูสับ ดมข้าว เผ็ด เค็ม ไม่หวาน ผลิตวันต่อวัน ไม่ใส่วัตถุกันเสีย ของแท้จากบริษัท ราคา 169.00 บาท</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4AxOqM1Q5R</t>
+          <t>https://s.shopee.co.th/3LOHqo8diW</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mhivoyzzzqird0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98z-lswcqt8y4gxp59.webp</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>done 2026-06-30 05:40</t>
+          <t>done 2026-06-30 05:41</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>น้ำพริกผัดหมูสับ ดมข้าว เผ็ด เค็ม ไม่หวาน ผลิตวันต่อวัน ไม่ใส่วัตถุกันเสีย ของแท้จากบริษัท ราคา 169.00 บาท</t>
+          <t>ปลาหมึกแห้ง ปลาหมึกแพไข่ ไซส์กลาง ไม่เค็มมาก ตากสดใหม่ รับประกันความอร่อย ราคา 129.00 บาท</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3LOHqo8diW</t>
+          <t>https://s.shopee.co.th/5q5alcgJru</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98z-lswcqt8y4gxp59.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-22110-pkze82odovjv1f.webp</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -3686,21 +3680,21 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ปลาหมึกแห้ง ปลาหมึกแพไข่ ไซส์กลาง ไม่เค็มมาก ตากสดใหม่ รับประกันความอร่อย ราคา 129.00 บาท</t>
+          <t>อุดมสุข น้ำพริกปลากะพง น้ำพริกคลีน น้ำพริกคีโต น้ำพริกเพื่อสุขภาพ ไม่ใส่ผงชูรส อาหารคลีน ราคา 169.00 บาท</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5q5alcgJru</t>
+          <t>https://s.shopee.co.th/5Apw2Yaqds</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-22110-pkze82odovjv1f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mk5i7m83jh1fa8.webp</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -3711,21 +3705,21 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>อุดมสุข น้ำพริกปลากะพง น้ำพริกคลีน น้ำพริกคีโต น้ำพริกเพื่อสุขภาพ ไม่ใส่ผงชูรส อาหารคลีน ราคา 169.00 บาท</t>
+          <t>มัทฉะ Kanbayashi Shunsho Usucha Aya no Mori อายะ โนะ โมริ 20g/40g Uji matcha【ส่งตรงจากญี่ปุ่น】 ราคา 1451.00 บาท</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5Apw2Yaqds</t>
+          <t>https://s.shopee.co.th/2Vp8nSwIA9</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mk5i7m83jh1fa8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mj8j4x9o8jd27f.webp</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -3736,439 +3730,414 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>มัทฉะ Kanbayashi Shunsho Usucha Aya no Mori อายะ โนะ โมริ 20g/40g Uji matcha【ส่งตรงจากญี่ปุ่น】 ราคา 1451.00 บาท</t>
+          <t>ใหม่!เซาปิ่งเปี๊ยะนุ่มลาวา สูตรเยาวราช 15 ปี ตัวแป้งทำจากมันเทศ เก็บได้นานเดือน อุ่นเวฟทานได้เรื่อยๆ</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2Vp8nSwIA9</t>
+          <t>https://s.shopee.co.th/6AiH6i2ekD</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mj8j4x9o8jd27f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mokxodhqmebkc8.webp</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>฿225</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>done 2026-06-30 05:41</t>
+          <t>done 2026-07-16 22:01</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>ใหม่!เซาปิ่งเปี๊ยะนุ่มลาวา สูตรเยาวราช 15 ปี ตัวแป้งทำจากมันเทศ เก็บได้นานเดือน อุ่นเวฟทานได้เรื่อยๆ</t>
+          <t>อึ่งไข่ฝนแรก ❗️พร้อมส่ง อึ่งไข่แช่แข็ง 📍อึ่งไข่ฝนแรกล็อตสุดท้ายของปีนี้</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6AiH6i2ekD</t>
+          <t>https://s.shopee.co.th/1gFrkRMbd1</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mokxodhqmebkc8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m8x3w0uh4ci73e.webp</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>฿225</t>
+          <t>฿1600</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>done 2026-07-16 22:01</t>
+          <t>done 2026-07-17 08:23</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>อึ่งไข่ฝนแรก ❗️พร้อมส่ง อึ่งไข่แช่แข็ง 📍อึ่งไข่ฝนแรกล็อตสุดท้ายของปีนี้</t>
+          <t>🔥 แคบหมูกึ่งสำเร็จรูป (ติดมัน) Pig a Pop แคบหมูแบบทอดเอง แคบหมูป๊อป แคบหมู แคปหมู</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1gFrkRMbd1</t>
+          <t>https://s.shopee.co.th/8fPc5JDYYT</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m8x3w0uh4ci73e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mib2ub5p89og02.webp</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>฿1600</t>
+          <t>฿90</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>done 2026-07-17 08:23</t>
+          <t>done 2026-07-17 19:39</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>🔥 แคบหมูกึ่งสำเร็จรูป (ติดมัน) Pig a Pop แคบหมูแบบทอดเอง แคบหมูป๊อป แคบหมู แคปหมู</t>
+          <t>ปลาหมึกแห้ง ปลาหมึกแพไข่ ไซส์กลาง ไม่เค็มมาก ตากสดใหม่ รับประกันความอร่อย</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8fPc5JDYYT</t>
+          <t>https://s.shopee.co.th/17dlNuzzw</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mib2ub5p89og02.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134201-22110-pkze82odovjv1f.webp</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>฿90</t>
-        </is>
-      </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>done 2026-07-17 19:39</t>
+          <t>฿129</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>ปลาหมึกแห้ง ปลาหมึกแพไข่ ไซส์กลาง ไม่เค็มมาก ตากสดใหม่ รับประกันความอร่อย</t>
+          <t>Chocolate Brownie Bite ช็อกโกแลตบราวนี่ไบท์ บราวนี่หน้าฟิล์ม</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/17dlNuzzw</t>
+          <t>https://s.shopee.co.th/1VwRY8x3aK</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134201-22110-pkze82odovjv1f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-23030-bggj3q1eovovda.webp</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>฿129</t>
+          <t>฿119</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Chocolate Brownie Bite ช็อกโกแลตบราวนี่ไบท์ บราวนี่หน้าฟิล์ม</t>
+          <t>ไข่ไก่เบอร์ 2 สดจากฟาร์ม 🥚 คัดพิเศษ ไข่ใหม่ทุกวัน</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1VwRY8x3aK</t>
+          <t>https://s.shopee.co.th/9Uyj4qWrbx</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-23030-bggj3q1eovovda.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mnkys1a0ddzcce.webp</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>฿119</t>
+          <t>฿80</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>ไข่ไก่เบอร์ 2 สดจากฟาร์ม 🥚 คัดพิเศษ ไข่ใหม่ทุกวัน</t>
+          <t>น้ำพริกแห้งปลาสลิดโรยข้าว รสผัดพริกขิง รสสมุนไพร รสน้ำพริกนรก แบบซอง ขนาด 100 กรัม 3 รสชาติ 1 ซอง Zalidpordeekum</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9Uyj4qWrbx</t>
+          <t>https://s.shopee.co.th/9pbZTSdhtH</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mnkys1a0ddzcce.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m863k6w28arga0.webp</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>฿80</t>
+          <t>฿160</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>น้ำพริกแห้งปลาสลิดโรยข้าว รสผัดพริกขิง รสสมุนไพร รสน้ำพริกนรก แบบซอง ขนาด 100 กรัม 3 รสชาติ 1 ซอง Zalidpordeekum</t>
+          <t>(แพ็ค 24 ซอง) Muek Groob หมึกกรุบ เส้นบุกปรุงรสหม่าล่า (เลือกรสชาติได้)</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9pbZTSdhtH</t>
+          <t>https://s.shopee.co.th/4Va37fQGTa</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m863k6w28arga0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0t-mbotiunlm1cj35.webp</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>฿160</t>
+          <t>฿502</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>(แพ็ค 24 ซอง) Muek Groob หมึกกรุบ เส้นบุกปรุงรสหม่าล่า (เลือกรสชาติได้)</t>
+          <t>น้ำพริกแซลมอนไข่เค็มคลีน ไม่มัน ไม่ใส่ผงชูรส ไม่ใส่สารกันเสีย ขนาด 150 กรัม</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4Va37fQGTa</t>
+          <t>https://s.shopee.co.th/902STwG4qp</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0t-mbotiunlm1cj35.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mkc4ypl093wg43.webp</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>฿502</t>
+          <t>฿150</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>น้ำพริกแซลมอนไข่เค็มคลีน ไม่มัน ไม่ใส่ผงชูรส ไม่ใส่สารกันเสีย ขนาด 150 กรัม</t>
+          <t>กุ้งขาวตัวใหญ่ๆ ไซส์25-35ตัวโล กุ้งสดๆแล้วนำมาแช่แข็ง ขายแพ็คละ 1กิโลกรัม เป็นกุ้งสดๆและนำไปแช่แข็ง</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/902STwG4qp</t>
+          <t>https://s.shopee.co.th/5ApjuteugA</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mkc4ypl093wg43.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m866iuk5c8e4b8.webp</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>฿150</t>
+          <t>฿300</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>กุ้งขาวตัวใหญ่ๆ ไซส์25-35ตัวโล กุ้งสดๆแล้วนำมาแช่แข็ง ขายแพ็คละ 1กิโลกรัม เป็นกุ้งสดๆและนำไปแช่แข็ง</t>
+          <t>กาแฟดำเพื่อสุขภาพ ไม่มีน้ำตาล คั่วสด บดละเอียด ผงสกัดกาแฟละลายน้ำร้อนทันที พร้อมดื่ม Healthy Black Coffee | ร้านกาแฟ 89</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5ApjuteugA</t>
+          <t>https://s.shopee.co.th/AAEPs5TAKT</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m866iuk5c8e4b8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98r-ly99vph2c04pdc.webp</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>฿300</t>
+          <t>฿99</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>กาแฟดำเพื่อสุขภาพ ไม่มีน้ำตาล คั่วสด บดละเอียด ผงสกัดกาแฟละลายน้ำร้อนทันที พร้อมดื่ม Healthy Black Coffee | ร้านกาแฟ 89</t>
+          <t>น้ำมันมรกต 1 ลิตร ยกลัง 12 ขวด สินค้าส่งตรงจากโรงงาน (1 คำสั่งซื้อ 1 ลัง) ต้องการมากกว่า 1 ให้แยกคำสั่งซื้อ</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AAEPs5TAKT</t>
+          <t>https://s.shopee.co.th/2LVYXh5iWf</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98r-ly99vph2c04pdc.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98u-lnfj2bxeyxioc3.webp</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>฿99</t>
+          <t>฿822</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>น้ำมันมรกต 1 ลิตร ยกลัง 12 ขวด สินค้าส่งตรงจากโรงงาน (1 คำสั่งซื้อ 1 ลัง) ต้องการมากกว่า 1 ให้แยกคำสั่งซื้อ</t>
+          <t>น้ำพริกหมูกระจกมะเดี่ยว วับวาว รสต้มยำ ชิ้นใหญ่ เต็มคำ แซ่บ เปรี้ยวเผ็ดสะใจ มี2ขนาด 100g./400g.</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2LVYXh5iWf</t>
+          <t>https://s.shopee.co.th/8KmlgitbG8</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98u-lnfj2bxeyxioc3.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mnmij2prwhl2a7.webp</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>฿822</t>
+          <t>฿175</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>น้ำพริกหมูกระจกมะเดี่ยว วับวาว รสต้มยำ ชิ้นใหญ่ เต็มคำ แซ่บ เปรี้ยวเผ็ดสะใจ มี2ขนาด 100g./400g.</t>
+          <t>ทุเรียนหมอนทอง คัดพิเศษ กล่องใหญ่ 3.5 กก.</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8KmlgitbG8</t>
+          <t>https://s.shopee.co.th/902STwyckb</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mnmij2prwhl2a7.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/f8fb32659a3650ce0dcc468f645e65be.webp</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>฿175</t>
+          <t>฿3700</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>ทุเรียนหมอนทอง คัดพิเศษ กล่องใหญ่ 3.5 กก.</t>
+          <t>มัทฉะ Kanbayashi Shunsho Usucha Aya no Mori อายะ โนะ โมริ 20g/40g Uji matcha【ส่งตรงจากญี่ปุ่น】</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/902STwyckb</t>
+          <t>https://s.shopee.co.th/AAEPs672Qs</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/f8fb32659a3650ce0dcc468f645e65be.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mj8j4x9o8jd27f.webp</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>฿3700</t>
+          <t>฿1451</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>มัทฉะ Kanbayashi Shunsho Usucha Aya no Mori อายะ โนะ โมริ 20g/40g Uji matcha【ส่งตรงจากญี่ปุ่น】</t>
+          <t>ระฆังทองน้ำปลาหวาน องค์พระปฐมเจดีย์</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AAEPs672Qs</t>
+          <t>https://s.shopee.co.th/gNKYdqLZf</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mj8j4x9o8jd27f.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/03ce1f8bce1154adcaab44a6dce2438a.webp</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
-        <is>
-          <t>฿1451</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="n">
-        <v>36</v>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>ระฆังทองน้ำปลาหวาน องค์พระปฐมเจดีย์</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/gNKYdqLZf</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>https://down-bs-th.img.susercontent.com/03ce1f8bce1154adcaab44a6dce2438a.webp</t>
-        </is>
-      </c>
-      <c r="F144" t="inlineStr">
         <is>
           <t>฿150</t>
         </is>

</xml_diff>